<commit_message>
Mise à jour du dépôt distant -
</commit_message>
<xml_diff>
--- a/database/datas-maternelle.xlsx
+++ b/database/datas-maternelle.xlsx
@@ -2,6 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
+  <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="O2XG4dl14fQAKlO0/hKvWGNqjnnWucpkY87cTmye/fhps0mMHaCLJWj5/ShghI3ULcBD6XpAVysU/oI6shUhpg==" workbookSaltValue="XbBWOJCXvcjAByP9rRIcHA==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
@@ -26427,13 +26428,13 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2" disablePrompts="0">
-        <x14:dataValidation xr:uid="{91D87F96-C87F-4266-B687-44EBEA05306F}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{39379799-C1C3-4BF7-93F4-F001C7A260C0}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>"1ère,2ème,3ème"</xm:f>
           </x14:formula1>
           <xm:sqref>N8:N1021 N1022 N1023 N1024 N1025</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{A5B1E94B-5FA6-4C1C-AEC4-57D243829267}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{64A8627C-9691-4B86-8946-7C61ECD1A015}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>"M,F"</xm:f>
           </x14:formula1>

</xml_diff>